<commit_message>
editable layout page on feedback sheet
</commit_message>
<xml_diff>
--- a/functional_tests/fixtures/dummy_grades.xlsx
+++ b/functional_tests/fixtures/dummy_grades.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Grades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grades" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat(assessment_feedback): infer grade subdivisions and dynamically recalculate cohort settings - Remove redundant global "Grade Band Subdivision" dropdown from the confirmation page (confirm.html) since subdivisions are auto-detected from spreadsheet values. - Add `data-subdivision` HTML attribute to individual category rubric panels in the template to track their specific subdivision. - Refactor Javascript helpers to read the subdivision per-panel and correctly pass it during rubric band rendering triggers. - Update server-side confirmation handler (`confirm_mappings` view) to dynamically recalculate the global cohort subdivision using the most common subdivision among all active grade categories. - Add comprehensive Django unit test to verify global cohort subdivision recalculation on form submission. - Update technical implementation logs in walkthrough.md.
</commit_message>
<xml_diff>
--- a/functional_tests/fixtures/dummy_grades.xlsx
+++ b/functional_tests/fixtures/dummy_grades.xlsx
@@ -1,34 +1,140 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Backup Drive\Documents\django-apps\feedback_dl\functional_tests\fixtures\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96C7B9CF-2B33-4DD2-A31F-B0171F868C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Grades" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+  <si>
+    <t>Student Name</t>
+  </si>
+  <si>
+    <t>Student ID</t>
+  </si>
+  <si>
+    <t>Design /30</t>
+  </si>
+  <si>
+    <t>Design Comments</t>
+  </si>
+  <si>
+    <t>Implementation /40</t>
+  </si>
+  <si>
+    <t>Implementation Comments</t>
+  </si>
+  <si>
+    <t>Testing /30</t>
+  </si>
+  <si>
+    <t>Testing Comments</t>
+  </si>
+  <si>
+    <t>Alice Smith</t>
+  </si>
+  <si>
+    <t>10001</t>
+  </si>
+  <si>
+    <t>Excellent software design, very modular.</t>
+  </si>
+  <si>
+    <t>Clean implementation with solid patterns.</t>
+  </si>
+  <si>
+    <t>Good coverage, though missing edge cases.</t>
+  </si>
+  <si>
+    <t>Bob Jones</t>
+  </si>
+  <si>
+    <t>10002</t>
+  </si>
+  <si>
+    <t>Adequate design, but lacks clean abstraction.</t>
+  </si>
+  <si>
+    <t>Some duplicate blocks observed, refactoring needed.</t>
+  </si>
+  <si>
+    <t>Minimal unit testing, several gaps.</t>
+  </si>
+  <si>
+    <t>Charlie Brown</t>
+  </si>
+  <si>
+    <t>10003</t>
+  </si>
+  <si>
+    <t>Masterclass design, highly maintainable.</t>
+  </si>
+  <si>
+    <t>Production-grade codebase, well styled.</t>
+  </si>
+  <si>
+    <t>Exhaustive tests covering extreme boundary limits.</t>
+  </si>
+  <si>
+    <t>High 2:1</t>
+  </si>
+  <si>
+    <t>Low 2:2</t>
+  </si>
+  <si>
+    <t>Mid 1st</t>
+  </si>
+  <si>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>3rd</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,81 +152,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,162 +456,125 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Student Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Student ID</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Design /30</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Design Comments</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Implementation /40</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Implementation Comments</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Testing /30</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Testing Comments</t>
-        </is>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Alice Smith</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>10001</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2">
         <v>24</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Excellent software design, very modular.</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2">
         <v>35</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Clean implementation with solid patterns.</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
         <v>25</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Good coverage, though missing edge cases.</t>
-        </is>
-      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bob Jones</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>10002</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
         <v>18</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Adequate design, but lacks clean abstraction.</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3">
         <v>28</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Some duplicate blocks observed, refactoring needed.</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Minimal unit testing, several gaps.</t>
-        </is>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Charlie Brown</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10003</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4">
         <v>28</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Masterclass design, highly maintainable.</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4">
         <v>38</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Production-grade codebase, well styled.</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Exhaustive tests covering extreme boundary limits.</t>
-        </is>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="1" t="str">
+        <f>"2:2"</f>
+        <v>2:2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
styled rubric mapping tables
</commit_message>
<xml_diff>
--- a/functional_tests/fixtures/dummy_grades.xlsx
+++ b/functional_tests/fixtures/dummy_grades.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Backup Drive\Documents\django-apps\feedback_dl\functional_tests\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96C7B9CF-2B33-4DD2-A31F-B0171F868C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682124AF-CFC2-4572-AFEB-D094CA8E1A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7110" yWindow="5520" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grades" sheetId="1" r:id="rId1"/>
@@ -47,15 +47,9 @@
     <t>Design Comments</t>
   </si>
   <si>
-    <t>Implementation /40</t>
-  </si>
-  <si>
     <t>Implementation Comments</t>
   </si>
   <si>
-    <t>Testing /30</t>
-  </si>
-  <si>
     <t>Testing Comments</t>
   </si>
   <si>
@@ -117,6 +111,12 @@
   </si>
   <si>
     <t>3rd</t>
+  </si>
+  <si>
+    <t>Implementation (40)</t>
+  </si>
+  <si>
+    <t>Testing 30</t>
   </si>
 </sst>
 </file>
@@ -474,103 +474,103 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
       <c r="I1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2">
         <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
         <v>23</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E3">
         <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E4">
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I4" s="1" t="str">
         <f>"2:2"</f>

</xml_diff>

<commit_message>
feat: add information category type for non-mark columns in assessment_feedback - Implemented keyword-based heuristics to auto-detect non-mark numeric columns (like "Max Load", "Time") on upload and automatically extract their units (e.g. "N", "kg"). - Added a visible "Type" dropdown in the confirm mapping page with choices (Mark, Rubric grade, Information data). - Implemented responsive JavaScript to hide/disable max marks, unit text inputs, and rubric panels conditionally based on selected column type. - Updated scoring context builders to exclude information columns from overall score, percentages, UK grade thresholds, and radar/histogram calculations. - Modified feedback sheet templates to render information categories as "Label: value unit" without denominators or grade bands. - Added comprehensive unit tests in tests.py covering auto-detection, validation, layout rendering, and scoring/radar chart exclusions. - Checked off the feature task inside ToDo.md.
</commit_message>
<xml_diff>
--- a/functional_tests/fixtures/dummy_grades.xlsx
+++ b/functional_tests/fixtures/dummy_grades.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Backup Drive\Documents\django-apps\feedback_dl\functional_tests\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682124AF-CFC2-4572-AFEB-D094CA8E1A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC723BE-C362-4654-AFEE-742FAAE09DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7110" yWindow="5520" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="855" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grades" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Student Name</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>Testing 30</t>
+  </si>
+  <si>
+    <t>Max Load (N)</t>
   </si>
 </sst>
 </file>
@@ -457,10 +460,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -488,8 +491,11 @@
       <c r="I1" t="s">
         <v>24</v>
       </c>
+      <c r="J1" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -517,8 +523,11 @@
       <c r="I2" t="s">
         <v>23</v>
       </c>
+      <c r="J2">
+        <v>234</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -546,8 +555,11 @@
       <c r="I3" t="s">
         <v>25</v>
       </c>
+      <c r="J3">
+        <v>111</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -575,6 +587,9 @@
       <c r="I4" s="1" t="str">
         <f>"2:2"</f>
         <v>2:2</v>
+      </c>
+      <c r="J4">
+        <v>543</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
populate email fields in send_emails file
</commit_message>
<xml_diff>
--- a/functional_tests/fixtures/dummy_grades.xlsx
+++ b/functional_tests/fixtures/dummy_grades.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Backup Drive\Documents\django-apps\feedback_dl\functional_tests\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC723BE-C362-4654-AFEE-742FAAE09DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B5C1DD-909F-4229-B10E-E206029FE855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="855" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grades" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Student Name</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Alice Smith</t>
   </si>
   <si>
-    <t>10001</t>
-  </si>
-  <si>
     <t>Excellent software design, very modular.</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>Bob Jones</t>
   </si>
   <si>
-    <t>10002</t>
-  </si>
-  <si>
     <t>Adequate design, but lacks clean abstraction.</t>
   </si>
   <si>
@@ -86,9 +80,6 @@
     <t>Charlie Brown</t>
   </si>
   <si>
-    <t>10003</t>
-  </si>
-  <si>
     <t>Masterclass design, highly maintainable.</t>
   </si>
   <si>
@@ -120,6 +111,12 @@
   </si>
   <si>
     <t>Max Load (N)</t>
+  </si>
+  <si>
+    <t>w12345678</t>
+  </si>
+  <si>
+    <t>12345687/1</t>
   </si>
 </sst>
 </file>
@@ -477,22 +474,22 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
       </c>
       <c r="I1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="J1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -500,28 +497,28 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C2">
         <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>35</v>
       </c>
       <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>10</v>
-      </c>
       <c r="I2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="J2">
         <v>234</v>
@@ -529,31 +526,31 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C3">
         <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E3">
         <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
         <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
       </c>
       <c r="J3">
         <v>111</v>
@@ -561,28 +558,28 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>87654321</v>
       </c>
       <c r="C4">
         <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E4">
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I4" s="1" t="str">
         <f>"2:2"</f>

</xml_diff>